<commit_message>
updated template referee blocks
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/PanAmProtocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/PanAmProtocol-A4.xlsx
@@ -1860,12 +1860,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:X125"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.85546875" customWidth="1"/>
     <col min="2" max="2" width="5.42578125" style="1" customWidth="1"/>
@@ -1890,7 +1890,7 @@
     <col min="25" max="25" width="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>20</v>
       </c>
@@ -1918,7 +1918,7 @@
       <c r="U1" s="96"/>
       <c r="V1" s="96"/>
     </row>
-    <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A2" s="35" t="s">
         <v>21</v>
       </c>
@@ -1945,7 +1945,7 @@
       <c r="T2" s="40"/>
       <c r="U2" s="40"/>
     </row>
-    <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A3" s="41" t="s">
         <v>22</v>
       </c>
@@ -1972,7 +1972,7 @@
       <c r="U3" s="45"/>
       <c r="V3" s="74"/>
     </row>
-    <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -1998,8 +1998,8 @@
       <c r="U4" s="124"/>
       <c r="V4" s="124"/>
     </row>
-    <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="6" customHeight="1" ns3:dyDescent="0.2"/>
+    <row r="6" spans="1:24" ht="15" customHeight="1" ns3:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="C6" s="8"/>
       <c r="H6" s="7"/>
@@ -2033,7 +2033,7 @@
       <c r="V6" s="105"/>
       <c r="X6"/>
     </row>
-    <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>40</v>
       </c>
@@ -2091,7 +2091,7 @@
       <c r="U7" s="106"/>
       <c r="V7" s="107"/>
     </row>
-    <row r="8" spans="1:24" s="22" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" s="22" customFormat="1" ht="7.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A8" s="46"/>
       <c r="B8" s="46"/>
       <c r="C8" s="46"/>
@@ -2104,7 +2104,7 @@
       <c r="J8" s="47"/>
       <c r="K8" s="48"/>
     </row>
-    <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="21.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A9" s="49" t="s">
         <v>82</v>
       </c>
@@ -2131,7 +2131,7 @@
       <c r="V9" s="77"/>
       <c r="X9"/>
     </row>
-    <row r="10" spans="1:24" s="22" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" s="22" customFormat="1" ht="21.2" customHeight="1" ns3:dyDescent="0.2">
       <c r="A10" s="81" t="s">
         <v>2</v>
       </c>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="V10" s="109"/>
     </row>
-    <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="24.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="B11"/>
       <c r="G11"/>
       <c r="H11"/>
@@ -2213,13 +2213,13 @@
       <c r="W11"/>
       <c r="X11"/>
     </row>
-    <row r="12" spans="1:24" s="32" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" s="32" customFormat="1" ht="15" ns3:dyDescent="0.25">
       <c r="A12" s="32" t="s">
         <v>63</v>
       </c>
       <c r="J12" s="33"/>
     </row>
-    <row r="13" spans="1:24" s="32" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" s="32" customFormat="1" ht="6.75" customHeight="1" ns3:dyDescent="0.25">
       <c r="A13" s="53"/>
       <c r="B13" s="53"/>
       <c r="C13" s="53"/>
@@ -2243,7 +2243,7 @@
       <c r="U13" s="59"/>
       <c r="V13" s="59"/>
     </row>
-    <row r="14" spans="1:24" s="71" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" s="71" customFormat="1" ht="12" ns3:dyDescent="0.2">
       <c r="A14" s="62" t="s">
         <v>71</v>
       </c>
@@ -2290,7 +2290,7 @@
       <c r="V14" s="70"/>
       <c r="X14" s="64"/>
     </row>
-    <row r="15" spans="1:24" s="52" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" s="52" customFormat="1" ns3:dyDescent="0.2">
       <c r="A15" s="54" t="s">
         <v>56</v>
       </c>
@@ -2337,11 +2337,11 @@
       <c r="V15" s="56"/>
       <c r="X15" s="56"/>
     </row>
-    <row r="16" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" ht="6" customHeight="1" ns3:dyDescent="0.2">
       <c r="C16" s="123"/>
       <c r="D16" s="123"/>
     </row>
-    <row r="17" spans="1:24" s="13" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" s="13" customFormat="1" ht="20.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A17" s="113" t="s">
         <v>47</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="16.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A18" s="113"/>
       <c r="B18" s="113"/>
       <c r="C18" s="122"/>
@@ -2410,7 +2410,7 @@
       <c r="V18" s="16"/>
       <c r="W18"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ns3:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="91"/>
       <c r="D19" s="1"/>
@@ -2433,7 +2433,7 @@
       <c r="V19" s="12"/>
       <c r="X19"/>
     </row>
-    <row r="20" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="13.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="25" t="s">
         <v>50</v>
@@ -2470,7 +2470,7 @@
       <c r="V20" s="78"/>
       <c r="X20"/>
     </row>
-    <row r="21" spans="1:24" s="18" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" s="18" customFormat="1" ht="12.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A21" s="19"/>
       <c r="B21" s="24"/>
       <c r="E21" s="17"/>
@@ -2480,7 +2480,7 @@
       <c r="Q21" s="19"/>
       <c r="V21" s="75"/>
     </row>
-    <row r="22" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" ht="17.45" customHeight="1" ns3:dyDescent="0.2">
       <c r="A22" s="94" t="s">
         <v>69</v>
       </c>
@@ -2504,7 +2504,7 @@
       <c r="W22"/>
       <c r="X22"/>
     </row>
-    <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="13.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A23" s="94"/>
       <c r="B23" s="94"/>
       <c r="C23" s="26" t="s">
@@ -2537,7 +2537,7 @@
       <c r="W23"/>
       <c r="X23"/>
     </row>
-    <row r="24" spans="1:24" s="18" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:24" s="18" customFormat="1" ht="11.25" ns3:dyDescent="0.2">
       <c r="B24" s="19"/>
       <c r="F24" s="15"/>
       <c r="G24" s="93"/>
@@ -2550,7 +2550,7 @@
       <c r="S24" s="19"/>
       <c r="V24" s="75"/>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" ns3:dyDescent="0.2">
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="H25" s="2"/>
@@ -2562,314 +2562,314 @@
       <c r="S25" s="1"/>
       <c r="T25" s="12"/>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" ns3:dyDescent="0.2">
       <c r="F26" s="1"/>
       <c r="U26" s="12"/>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:24" ns3:dyDescent="0.2">
       <c r="F27" s="1"/>
       <c r="U27" s="12"/>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:24" ns3:dyDescent="0.2">
       <c r="F28" s="1"/>
       <c r="U28" s="12"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:24" ns3:dyDescent="0.2">
       <c r="F29" s="1"/>
       <c r="U29" s="12"/>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" ns3:dyDescent="0.2">
       <c r="F30" s="1"/>
       <c r="U30" s="12"/>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:24" ns3:dyDescent="0.2">
       <c r="D31" s="20"/>
       <c r="E31" s="20"/>
       <c r="F31" s="1"/>
       <c r="U31" s="12"/>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:24" ns3:dyDescent="0.2">
       <c r="F32" s="1"/>
       <c r="U32" s="12"/>
     </row>
-    <row r="33" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="33" spans="6:21" ns3:dyDescent="0.2">
       <c r="F33" s="1"/>
       <c r="U33" s="12"/>
     </row>
-    <row r="34" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="34" spans="6:21" ns3:dyDescent="0.2">
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="35" spans="6:21" ns3:dyDescent="0.2">
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="36" spans="6:21" ns3:dyDescent="0.2">
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="37" spans="6:21" ns3:dyDescent="0.2">
       <c r="F37" s="1"/>
     </row>
-    <row r="38" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="38" spans="6:21" ns3:dyDescent="0.2">
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="39" spans="6:21" ns3:dyDescent="0.2">
       <c r="F39" s="1"/>
     </row>
-    <row r="40" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="40" spans="6:21" ns3:dyDescent="0.2">
       <c r="F40" s="1"/>
     </row>
-    <row r="41" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="41" spans="6:21" ns3:dyDescent="0.2">
       <c r="F41" s="1"/>
     </row>
-    <row r="42" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="42" spans="6:21" ns3:dyDescent="0.2">
       <c r="F42" s="1"/>
     </row>
-    <row r="43" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="43" spans="6:21" ns3:dyDescent="0.2">
       <c r="F43" s="1"/>
     </row>
-    <row r="44" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="44" spans="6:21" ns3:dyDescent="0.2">
       <c r="F44" s="1"/>
     </row>
-    <row r="45" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="45" spans="6:21" ns3:dyDescent="0.2">
       <c r="F45" s="1"/>
     </row>
-    <row r="46" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="46" spans="6:21" ns3:dyDescent="0.2">
       <c r="F46" s="1"/>
     </row>
-    <row r="47" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="47" spans="6:21" ns3:dyDescent="0.2">
       <c r="F47" s="1"/>
     </row>
-    <row r="48" spans="6:21" x14ac:dyDescent="0.2">
+    <row r="48" spans="6:21" ns3:dyDescent="0.2">
       <c r="F48" s="1"/>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="6:6" ns3:dyDescent="0.2">
       <c r="F49" s="1"/>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="6:6" ns3:dyDescent="0.2">
       <c r="F50" s="1"/>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="6:6" ns3:dyDescent="0.2">
       <c r="F51" s="1"/>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="6:6" ns3:dyDescent="0.2">
       <c r="F52" s="1"/>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="6:6" ns3:dyDescent="0.2">
       <c r="F53" s="1"/>
     </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="6:6" ns3:dyDescent="0.2">
       <c r="F54" s="1"/>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="6:6" ns3:dyDescent="0.2">
       <c r="F55" s="1"/>
     </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="6:6" ns3:dyDescent="0.2">
       <c r="F56" s="1"/>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="6:6" ns3:dyDescent="0.2">
       <c r="F57" s="1"/>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="6:6" ns3:dyDescent="0.2">
       <c r="F58" s="1"/>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="6:6" ns3:dyDescent="0.2">
       <c r="F59" s="1"/>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="6:6" ns3:dyDescent="0.2">
       <c r="F60" s="1"/>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="6:6" ns3:dyDescent="0.2">
       <c r="F61" s="1"/>
     </row>
-    <row r="62" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="6:6" ns3:dyDescent="0.2">
       <c r="F62" s="1"/>
     </row>
-    <row r="63" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="6:6" ns3:dyDescent="0.2">
       <c r="F63" s="1"/>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="6:6" ns3:dyDescent="0.2">
       <c r="F64" s="1"/>
     </row>
-    <row r="65" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="6:6" ns3:dyDescent="0.2">
       <c r="F65" s="1"/>
     </row>
-    <row r="66" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="6:6" ns3:dyDescent="0.2">
       <c r="F66" s="1"/>
     </row>
-    <row r="67" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="6:6" ns3:dyDescent="0.2">
       <c r="F67" s="1"/>
     </row>
-    <row r="68" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="6:6" ns3:dyDescent="0.2">
       <c r="F68" s="1"/>
     </row>
-    <row r="69" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="6:6" ns3:dyDescent="0.2">
       <c r="F69" s="1"/>
     </row>
-    <row r="70" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="6:6" ns3:dyDescent="0.2">
       <c r="F70" s="1"/>
     </row>
-    <row r="71" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="6:6" ns3:dyDescent="0.2">
       <c r="F71" s="1"/>
     </row>
-    <row r="72" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="6:6" ns3:dyDescent="0.2">
       <c r="F72" s="1"/>
     </row>
-    <row r="73" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="6:6" ns3:dyDescent="0.2">
       <c r="F73" s="1"/>
     </row>
-    <row r="74" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="6:6" ns3:dyDescent="0.2">
       <c r="F74" s="1"/>
     </row>
-    <row r="75" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="6:6" ns3:dyDescent="0.2">
       <c r="F75" s="1"/>
     </row>
-    <row r="76" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="6:6" ns3:dyDescent="0.2">
       <c r="F76" s="1"/>
     </row>
-    <row r="77" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="6:6" ns3:dyDescent="0.2">
       <c r="F77" s="1"/>
     </row>
-    <row r="78" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="6:6" ns3:dyDescent="0.2">
       <c r="F78" s="1"/>
     </row>
-    <row r="79" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="6:6" ns3:dyDescent="0.2">
       <c r="F79" s="1"/>
     </row>
-    <row r="80" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="6:6" ns3:dyDescent="0.2">
       <c r="F80" s="1"/>
     </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="6:6" ns3:dyDescent="0.2">
       <c r="F81" s="1"/>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="6:6" ns3:dyDescent="0.2">
       <c r="F82" s="1"/>
     </row>
-    <row r="83" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="6:6" ns3:dyDescent="0.2">
       <c r="F83" s="1"/>
     </row>
-    <row r="84" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="6:6" ns3:dyDescent="0.2">
       <c r="F84" s="1"/>
     </row>
-    <row r="85" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="6:6" ns3:dyDescent="0.2">
       <c r="F85" s="1"/>
     </row>
-    <row r="86" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="6:6" ns3:dyDescent="0.2">
       <c r="F86" s="1"/>
     </row>
-    <row r="87" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="6:6" ns3:dyDescent="0.2">
       <c r="F87" s="1"/>
     </row>
-    <row r="88" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="6:6" ns3:dyDescent="0.2">
       <c r="F88" s="1"/>
     </row>
-    <row r="89" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="6:6" ns3:dyDescent="0.2">
       <c r="F89" s="1"/>
     </row>
-    <row r="90" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="6:6" ns3:dyDescent="0.2">
       <c r="F90" s="1"/>
     </row>
-    <row r="91" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="6:6" ns3:dyDescent="0.2">
       <c r="F91" s="1"/>
     </row>
-    <row r="92" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="6:6" ns3:dyDescent="0.2">
       <c r="F92" s="1"/>
     </row>
-    <row r="93" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="6:6" ns3:dyDescent="0.2">
       <c r="F93" s="1"/>
     </row>
-    <row r="94" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="6:6" ns3:dyDescent="0.2">
       <c r="F94" s="1"/>
     </row>
-    <row r="95" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="6:6" ns3:dyDescent="0.2">
       <c r="F95" s="1"/>
     </row>
-    <row r="96" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="6:6" ns3:dyDescent="0.2">
       <c r="F96" s="1"/>
     </row>
-    <row r="97" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="6:6" ns3:dyDescent="0.2">
       <c r="F97" s="1"/>
     </row>
-    <row r="98" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="6:6" ns3:dyDescent="0.2">
       <c r="F98" s="1"/>
     </row>
-    <row r="99" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="6:6" ns3:dyDescent="0.2">
       <c r="F99" s="1"/>
     </row>
-    <row r="100" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="6:6" ns3:dyDescent="0.2">
       <c r="F100" s="1"/>
     </row>
-    <row r="101" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="6:6" ns3:dyDescent="0.2">
       <c r="F101" s="1"/>
     </row>
-    <row r="102" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="6:6" ns3:dyDescent="0.2">
       <c r="F102" s="1"/>
     </row>
-    <row r="103" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="6:6" ns3:dyDescent="0.2">
       <c r="F103" s="1"/>
     </row>
-    <row r="104" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="6:6" ns3:dyDescent="0.2">
       <c r="F104" s="1"/>
     </row>
-    <row r="105" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="6:6" ns3:dyDescent="0.2">
       <c r="F105" s="1"/>
     </row>
-    <row r="106" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="6:6" ns3:dyDescent="0.2">
       <c r="F106" s="1"/>
     </row>
-    <row r="107" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="6:6" ns3:dyDescent="0.2">
       <c r="F107" s="1"/>
     </row>
-    <row r="108" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="6:6" ns3:dyDescent="0.2">
       <c r="F108" s="1"/>
     </row>
-    <row r="109" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="6:6" ns3:dyDescent="0.2">
       <c r="F109" s="1"/>
     </row>
-    <row r="110" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="6:6" ns3:dyDescent="0.2">
       <c r="F110" s="1"/>
     </row>
-    <row r="111" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="6:6" ns3:dyDescent="0.2">
       <c r="F111" s="1"/>
     </row>
-    <row r="112" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="6:6" ns3:dyDescent="0.2">
       <c r="F112" s="1"/>
     </row>
-    <row r="113" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="6:6" ns3:dyDescent="0.2">
       <c r="F113" s="1"/>
     </row>
-    <row r="114" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="6:6" ns3:dyDescent="0.2">
       <c r="F114" s="1"/>
     </row>
-    <row r="115" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="6:6" ns3:dyDescent="0.2">
       <c r="F115" s="1"/>
     </row>
-    <row r="116" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="6:6" ns3:dyDescent="0.2">
       <c r="F116" s="1"/>
     </row>
-    <row r="117" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="6:6" ns3:dyDescent="0.2">
       <c r="F117" s="1"/>
     </row>
-    <row r="118" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="6:6" ns3:dyDescent="0.2">
       <c r="F118" s="1"/>
     </row>
-    <row r="119" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="6:6" ns3:dyDescent="0.2">
       <c r="F119" s="1"/>
     </row>
-    <row r="120" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="6:6" ns3:dyDescent="0.2">
       <c r="F120" s="1"/>
     </row>
-    <row r="121" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="6:6" ns3:dyDescent="0.2">
       <c r="F121" s="1"/>
     </row>
-    <row r="122" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="6:6" ns3:dyDescent="0.2">
       <c r="F122" s="1"/>
     </row>
-    <row r="123" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="6:6" ns3:dyDescent="0.2">
       <c r="F123" s="1"/>
     </row>
-    <row r="124" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="6:6" ns3:dyDescent="0.2">
       <c r="F124" s="1"/>
     </row>
-    <row r="125" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="6:6" ns3:dyDescent="0.2">
       <c r="F125" s="1"/>
     </row>
   </sheetData>
@@ -2913,24 +2913,24 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation showErrorMessage="1" sqref="K4 F23 C20 S18 S23 F20 C23 L20 S20 C17 L17 F18" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="H11:H13" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation showErrorMessage="1" sqref="K4 F23 C20 S18 S23 F20 C23 L20 S20 C17 L17 F18" ns2:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" ns2:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="H11:H13" ns2:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I8" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I8" ns2:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="www.federation.org" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="A4" r:id="rId2" display="records@federation.org" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="A3" ns4:id="rId1" display="www.federation.org" ns2:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A4" ns4:id="rId2" display="records@federation.org" ns2:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.31496062992125984" right="0.35433070866141736" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="70" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="70" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" ns4:id="rId3"/>
   <headerFooter alignWithMargins="0"/>
-  <legacyDrawing r:id="rId4"/>
+  <legacyDrawing ns4:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>